<commit_message>
feat(gbm-reader): improve numeric parsing for currency and percentage values
- Add _parse_num() helper function to handle currency ($), percentage (%), and dash (-) formatted values
- Replace repetitive float conversion logic with _parse_num() calls across read_nacional() function
- Replace repetitive float conversion logic with _parse_num() calls across read_usa() function
- Handle edge cases: None values, empty strings, "N/A", and negative currency amounts
- Update cash entry validation to use _parse_num() for consistent zero-value detection
- Update backend and frontend logs with latest application runtime data
- Add last_updates.json tracking file for data synchronization
- Consolidate numeric parsing to reduce code duplication and improve maintainability
</commit_message>
<xml_diff>
--- a/data/GI/gastos-ingresos.xlsx
+++ b/data/GI/gastos-ingresos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1624,6 +1624,34 @@
         <v>-602.76</v>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Uber</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>ingreso</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>105.56</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>